<commit_message>
Added average DSS confidence, fixes in submission form, and update docu
</commit_message>
<xml_diff>
--- a/docs/dss-matrix.xlsx
+++ b/docs/dss-matrix.xlsx
@@ -60,88 +60,88 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Item</t>
+          <t>Screening</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>item_type/details.item_types</t>
+          <t>details.uniform_branding</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>What type of item/s are you submitting?</t>
+          <t>Donation only: uniform or identifiable company/school/institutional branding?</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Top; Pants/Jeans; Dress; Jacket; Household textile; Fabric scraps; Other</t>
+          <t>Yes blocks Donation and recommends Upcycle or Recycle; No continues</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Condition</t>
+          <t>Item</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>condition</t>
+          <t>item_type/details.item_types</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Overall condition</t>
+          <t>What type of item/s are you submitting?</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Good; Minor damage; Heavily damaged</t>
+          <t>Donation excludes Fabric scraps. Recycle/Upcycle: Top; Pants/Jeans; Dress; Jacket; Household textile; Fabric scraps; Other</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Cleanliness</t>
+          <t>Condition</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>cleanliness</t>
+          <t>condition</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Is/are the item/s clean?</t>
+          <t>Overall condition</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Clean; Needs cleaning; Heavily soiled/contaminated</t>
+          <t>Good; Minor damage; Heavily damaged</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Fabric</t>
+          <t>Cleanliness</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>details.knows_fabric_type</t>
+          <t>cleanliness</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Do you know the fabric type?</t>
+          <t>Is/are the item/s clean?</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Yes; No</t>
+          <t>Donation blocks Heavily soiled/contaminated; other forms keep existing behavior</t>
         </is>
       </c>
     </row>
@@ -153,17 +153,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>details.fabric_types</t>
+          <t>details.knows_fabric_type</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>What is the fabric type?</t>
+          <t>Do you know the fabric type?</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Cotton/Linen; Polyester/nylon/acrylic; Viscose/Rayon; Blends; Coated/PPE; Wool/Silk; Other/user-defined</t>
+          <t>Yes; No</t>
         </is>
       </c>
     </row>
@@ -175,17 +175,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>details.custom_fabric_text</t>
+          <t>details.fabric_types</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>User-defined fabric text</t>
+          <t>What is the fabric type?</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Free text</t>
+          <t>Cotton/Linen; Polyester/nylon/acrylic; Viscose/Rayon; Blends; Coated/PPE; Wool/Silk; Other/user-defined</t>
         </is>
       </c>
     </row>
@@ -197,37 +197,103 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>details.fiber_composition</t>
+          <t>details.custom_fabric_text</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Main material/fiber composition</t>
+          <t>User-defined fabric text</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Cotton/natural; Polyester/synthetic; Blend; Wool/silk/delicate; Mixed/unknown</t>
+          <t>Free text</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>Fabric</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>details.fiber_composition</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Main material/fiber composition</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Cotton/natural; Polyester/synthetic; Blend; Wool/silk/delicate; Mixed/unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>Recovery</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>details.wearability</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Is the item still wearable or usable?</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Donation skips Recovery. Recycle/Upcycle disable and do not require/score when Fabric scraps is the only selected item type</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Recovery</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>details.repairability</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Is the item repairable?</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Donation skips Recovery. Recycle/Upcycle disable and do not require/score when Fabric scraps is the only selected item type</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Recovery</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
         <is>
           <t>details.contamination_level</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>Contamination level</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>Only if condition is minor/heavy damage</t>
         </is>
@@ -629,17 +695,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Wearability</t>
+          <t>Hard eligibility</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>Block</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Wearable as-is or minor repair</t>
+          <t>Blocks uniforms/branded institutional clothing, heavily damaged items, heavily soiled/contaminated items, and Fabric scraps</t>
         </is>
       </c>
     </row>
@@ -651,17 +717,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Cleanliness/contamination</t>
+          <t>Item choices</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Clean or washable only</t>
+          <t>Fabric scraps is removed from Donation item type choices</t>
         </is>
       </c>
     </row>
@@ -673,51 +739,51 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Damage/repair</t>
+          <t>Recovery Criteria</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>No damage or minor repairable damage</t>
+          <t>Donation form skips Recovery Criteria entirely</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Upcycle</t>
+          <t>Donation</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Repurposing potential</t>
+          <t>Wearability</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>20</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>High or medium</t>
+          <t>Wearable as-is or minor repair</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Upcycle</t>
+          <t>Donation</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Repairability/damage</t>
+          <t>Cleanliness/contamination</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -727,49 +793,137 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Repair/redesign can preserve material value</t>
+          <t>Clean or washable only</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Recycle</t>
+          <t>Donation</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Fabric/material signal</t>
+          <t>Damage/repair</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>17</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Identifiable recyclable fiber/material</t>
+          <t>No damage or minor repairable damage</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>All applicable Recovery forms</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Fabric scraps-only skip</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Normalize</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>When only Fabric scraps is selected, Wearability and Repairability are disabled, cleared, not required, and excluded from scoring normalization</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Upcycle</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Repurposing potential</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>High or medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Upcycle</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Repairability/damage</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Repair/redesign can preserve material value</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>Recycle</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Fabric/material signal</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Identifiable recyclable fiber/material</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Recycle</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
         <is>
           <t>Damage/contamination/trim</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>45</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>Material recovery fit without hazardous contamination</t>
         </is>
@@ -830,6 +984,30 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Donation uniform/branded clothing</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Block Donation only; store details.uniform_branding for DSS audit consistency</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Fabric scraps-only Recovery Criteria</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Disable Wearability and Repairability; submit null values and exclude their weights from scoring</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>